<commit_message>
tiktok upload first run
</commit_message>
<xml_diff>
--- a/videos.xlsx
+++ b/videos.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,16 +29,8 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C6500"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -48,11 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,12 +55,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -451,6 +435,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,23 +484,27 @@
           <t>Error / notes</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>TikTok link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>https://upload.wikimedia.org/wikipedia/commons/c/ce/Bodycam_Footage_Captures_LAPD_Officer_Beating_Trespassing_Man.webm</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>